<commit_message>
Added Account Scenario Tests
</commit_message>
<xml_diff>
--- a/src/main/resource/testdata/OpenCartRegUserTestData.xlsx
+++ b/src/main/resource/testdata/OpenCartRegUserTestData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MY_Selenium_POM\src\main\resource\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADF57588-FF4F-4508-9815-1DEF51A26083}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AE04EA9-8C9D-4C8B-9405-25002AFD936C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{7B1AA3E2-B494-4213-8E38-6CBE51FC50B4}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="56">
   <si>
     <t>Account Name</t>
   </si>
@@ -114,6 +114,96 @@
   </si>
   <si>
     <t>2</t>
+  </si>
+  <si>
+    <t>Creating New Contact</t>
+  </si>
+  <si>
+    <t>FirstName</t>
+  </si>
+  <si>
+    <t>LastName</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>Creating_Contact_Through_Automation</t>
+  </si>
+  <si>
+    <t>Department</t>
+  </si>
+  <si>
+    <t>Communications</t>
+  </si>
+  <si>
+    <t>Phone</t>
+  </si>
+  <si>
+    <t>This Contact is created By Selenium Automation Script</t>
+  </si>
+  <si>
+    <t>Lead Source</t>
+  </si>
+  <si>
+    <t>Phone Inquiry</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>EditingContactByClickingEditBtn</t>
+  </si>
+  <si>
+    <t>Mailing Street_c</t>
+  </si>
+  <si>
+    <t>Mailing State_c</t>
+  </si>
+  <si>
+    <t>Mailing City_c</t>
+  </si>
+  <si>
+    <t>Mailing Country_c</t>
+  </si>
+  <si>
+    <t>Mailing Zipcode_c</t>
+  </si>
+  <si>
+    <t>Language</t>
+  </si>
+  <si>
+    <t>English</t>
+  </si>
+  <si>
+    <t>Level</t>
+  </si>
+  <si>
+    <t>Tertiary</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>Editing Contact By Clicking Inline Btn</t>
+  </si>
+  <si>
+    <t>Home Phone</t>
+  </si>
+  <si>
+    <t>Other Phone</t>
+  </si>
+  <si>
+    <t>Assistant</t>
+  </si>
+  <si>
+    <t>Asst Phone</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>9876896543</t>
   </si>
 </sst>
 </file>
@@ -185,12 +275,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -525,16 +616,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D41DAC7C-D34E-4D5E-987A-8E1EB0CBFB48}">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30.7265625" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.90625" style="3" customWidth="1"/>
     <col min="3" max="3" width="22.26953125" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33" style="3" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="45.1796875" style="3" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="23.26953125" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.36328125" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="45" style="3" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.90625" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.26953125" style="3" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17.36328125" style="3" bestFit="1" customWidth="1"/>
@@ -687,6 +778,170 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8" s="2">
+        <v>9876543212</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="J9" s="2"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" s="2">
+        <v>93030</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="J10" s="2"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A12" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F12" s="2">
+        <v>9876896543</v>
+      </c>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added Lead,Contact and Account Scenario's
</commit_message>
<xml_diff>
--- a/src/main/resource/testdata/OpenCartRegUserTestData.xlsx
+++ b/src/main/resource/testdata/OpenCartRegUserTestData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MY_Selenium_POM\src\main\resource\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AE04EA9-8C9D-4C8B-9405-25002AFD936C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A640CDE0-11FC-4A30-8F9E-795E1F743A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{7B1AA3E2-B494-4213-8E38-6CBE51FC50B4}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="86">
   <si>
     <t>Account Name</t>
   </si>
@@ -204,13 +204,103 @@
   </si>
   <si>
     <t>9876896543</t>
+  </si>
+  <si>
+    <t>Creating New Lead</t>
+  </si>
+  <si>
+    <t>Company</t>
+  </si>
+  <si>
+    <t>Industry</t>
+  </si>
+  <si>
+    <t>Rating</t>
+  </si>
+  <si>
+    <t>Baymont</t>
+  </si>
+  <si>
+    <t>Creating_Lead_Through_Automation</t>
+  </si>
+  <si>
+    <t>Warm</t>
+  </si>
+  <si>
+    <t>This Lead is created By Selenium Automation Script</t>
+  </si>
+  <si>
+    <t>No.of Employee</t>
+  </si>
+  <si>
+    <t>Street</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>State</t>
+  </si>
+  <si>
+    <t>Pincode</t>
+  </si>
+  <si>
+    <t>Countrty</t>
+  </si>
+  <si>
+    <t>130</t>
+  </si>
+  <si>
+    <t>EditingLeadByClickingEditBtn</t>
+  </si>
+  <si>
+    <t>Mobile Phone</t>
+  </si>
+  <si>
+    <t>Website</t>
+  </si>
+  <si>
+    <t>Product Interest</t>
+  </si>
+  <si>
+    <t>SIC Code</t>
+  </si>
+  <si>
+    <t>Number Locations</t>
+  </si>
+  <si>
+    <t>Current Generator</t>
+  </si>
+  <si>
+    <t>Primary</t>
+  </si>
+  <si>
+    <t>9878654567</t>
+  </si>
+  <si>
+    <t>www.test.com</t>
+  </si>
+  <si>
+    <t>GC5000 series</t>
+  </si>
+  <si>
+    <t>test112</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>EditingLeadByClickingInlineEditBtn</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -229,6 +319,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -272,18 +370,21 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -616,7 +717,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D41DAC7C-D34E-4D5E-987A-8E1EB0CBFB48}">
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30.7265625" style="3" bestFit="1" customWidth="1"/>
@@ -626,10 +727,11 @@
     <col min="5" max="5" width="45.1796875" style="3" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="23.26953125" style="3" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="45" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.90625" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.6328125" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.26953125" style="3" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17.36328125" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="8.7265625" style="3"/>
+    <col min="11" max="11" width="10.1796875" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.7265625" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
@@ -942,11 +1044,194 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H14" s="2">
+        <v>987656789</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A16" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G16" s="2">
+        <v>93030</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="J17" s="1"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A18" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="J18" s="2"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A19" s="1" t="s">
         <v>19</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D18" r:id="rId1" xr:uid="{33FAECC2-53B2-4370-A4DF-0F34ABF4AD69}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>